<commit_message>
chore: BBS取得 2026-09-15 07:10
</commit_message>
<xml_diff>
--- a/bbs_log.xlsx
+++ b/bbs_log.xlsx
@@ -419,7 +419,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H524"/>
+  <dimension ref="A1:H530"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -16623,7 +16623,6 @@
           <t>キムとドMみい</t>
         </is>
       </c>
-      <c r="E515" t="inlineStr"/>
       <c r="F515" t="inlineStr">
         <is>
           <t>みんなで</t>
@@ -16634,7 +16633,6 @@
           <t>いじめて下さい</t>
         </is>
       </c>
-      <c r="H515" t="inlineStr"/>
     </row>
     <row r="516">
       <c r="A516" t="n">
@@ -16655,7 +16653,6 @@
           <t>タケ</t>
         </is>
       </c>
-      <c r="E516" t="inlineStr"/>
       <c r="F516" t="inlineStr">
         <is>
           <t>初めて</t>
@@ -16666,7 +16663,6 @@
           <t>来ました</t>
         </is>
       </c>
-      <c r="H516" t="inlineStr"/>
     </row>
     <row r="517">
       <c r="A517" t="n">
@@ -16687,7 +16683,6 @@
           <t>くれは</t>
         </is>
       </c>
-      <c r="E517" t="inlineStr"/>
       <c r="F517" t="inlineStr">
         <is>
           <t>今</t>
@@ -16698,7 +16693,6 @@
           <t>きました！</t>
         </is>
       </c>
-      <c r="H517" t="inlineStr"/>
     </row>
     <row r="518">
       <c r="A518" t="n">
@@ -16719,7 +16713,6 @@
           <t>キム、みー</t>
         </is>
       </c>
-      <c r="E518" t="inlineStr"/>
       <c r="F518" t="inlineStr">
         <is>
           <t>今</t>
@@ -16730,7 +16723,6 @@
           <t>きたたった</t>
         </is>
       </c>
-      <c r="H518" t="inlineStr"/>
     </row>
     <row r="519">
       <c r="A519" t="n">
@@ -16751,7 +16743,6 @@
           <t>ゆずきち</t>
         </is>
       </c>
-      <c r="E519" t="inlineStr"/>
       <c r="F519" t="inlineStr">
         <is>
           <t>今</t>
@@ -16762,7 +16753,6 @@
           <t>きたんご</t>
         </is>
       </c>
-      <c r="H519" t="inlineStr"/>
     </row>
     <row r="520">
       <c r="A520" t="n">
@@ -16783,7 +16773,6 @@
           <t>ゆう</t>
         </is>
       </c>
-      <c r="E520" t="inlineStr"/>
       <c r="F520" t="inlineStr">
         <is>
           <t>はじめて</t>
@@ -16794,7 +16783,6 @@
           <t>きました！</t>
         </is>
       </c>
-      <c r="H520" t="inlineStr"/>
     </row>
     <row r="521">
       <c r="A521" t="n">
@@ -16815,7 +16803,6 @@
           <t>ましゅ</t>
         </is>
       </c>
-      <c r="E521" t="inlineStr"/>
       <c r="F521" t="inlineStr">
         <is>
           <t>パチンコ</t>
@@ -16826,7 +16813,6 @@
           <t>まけちゃった</t>
         </is>
       </c>
-      <c r="H521" t="inlineStr"/>
     </row>
     <row r="522">
       <c r="A522" t="n">
@@ -16847,7 +16833,6 @@
           <t>りゅーちゃん、まな</t>
         </is>
       </c>
-      <c r="E522" t="inlineStr"/>
       <c r="F522" t="inlineStr">
         <is>
           <t>新規</t>
@@ -16858,7 +16843,6 @@
           <t>連れてきました</t>
         </is>
       </c>
-      <c r="H522" t="inlineStr"/>
     </row>
     <row r="523">
       <c r="A523" t="n">
@@ -16879,7 +16863,6 @@
           <t>ひがん</t>
         </is>
       </c>
-      <c r="E523" t="inlineStr"/>
       <c r="F523" t="inlineStr">
         <is>
           <t>ねむすぎ</t>
@@ -16890,7 +16873,6 @@
           <t>来たっちゃ</t>
         </is>
       </c>
-      <c r="H523" t="inlineStr"/>
     </row>
     <row r="524">
       <c r="A524" t="n">
@@ -16944,6 +16926,218 @@
         </is>
       </c>
     </row>
+    <row r="525">
+      <c r="A525" t="n">
+        <v>27775</v>
+      </c>
+      <c r="B525" t="inlineStr">
+        <is>
+          <t>2026-09-14</t>
+        </is>
+      </c>
+      <c r="C525" t="inlineStr">
+        <is>
+          <t>19:21:38</t>
+        </is>
+      </c>
+      <c r="D525" t="inlineStr">
+        <is>
+          <t>ひがん</t>
+        </is>
+      </c>
+      <c r="E525" t="inlineStr"/>
+      <c r="F525" t="inlineStr">
+        <is>
+          <t>ちいかわ観て</t>
+        </is>
+      </c>
+      <c r="G525" t="inlineStr">
+        <is>
+          <t>来ました♪</t>
+        </is>
+      </c>
+      <c r="H525" t="inlineStr"/>
+    </row>
+    <row r="526">
+      <c r="A526" t="n">
+        <v>27776</v>
+      </c>
+      <c r="B526" t="inlineStr">
+        <is>
+          <t>2026-09-14</t>
+        </is>
+      </c>
+      <c r="C526" t="inlineStr">
+        <is>
+          <t>19:22:11</t>
+        </is>
+      </c>
+      <c r="D526" t="inlineStr">
+        <is>
+          <t>bee</t>
+        </is>
+      </c>
+      <c r="E526" t="inlineStr"/>
+      <c r="F526" t="inlineStr">
+        <is>
+          <t>遊びに</t>
+        </is>
+      </c>
+      <c r="G526" t="inlineStr">
+        <is>
+          <t>来ましたブン♪</t>
+        </is>
+      </c>
+      <c r="H526" t="inlineStr"/>
+    </row>
+    <row r="527">
+      <c r="A527" t="n">
+        <v>27779</v>
+      </c>
+      <c r="B527" t="inlineStr">
+        <is>
+          <t>2026-09-14</t>
+        </is>
+      </c>
+      <c r="C527" t="inlineStr">
+        <is>
+          <t>19:57:51</t>
+        </is>
+      </c>
+      <c r="D527" t="inlineStr">
+        <is>
+          <t>ろくじ</t>
+        </is>
+      </c>
+      <c r="E527" t="inlineStr"/>
+      <c r="F527" t="inlineStr">
+        <is>
+          <t>飲みに</t>
+        </is>
+      </c>
+      <c r="G527" t="inlineStr">
+        <is>
+          <t>来ました！</t>
+        </is>
+      </c>
+      <c r="H527" t="inlineStr"/>
+    </row>
+    <row r="528">
+      <c r="A528" t="n">
+        <v>27780</v>
+      </c>
+      <c r="B528" t="inlineStr">
+        <is>
+          <t>2026-09-14</t>
+        </is>
+      </c>
+      <c r="C528" t="inlineStr">
+        <is>
+          <t>20:43:04</t>
+        </is>
+      </c>
+      <c r="D528" t="inlineStr">
+        <is>
+          <t>まみ</t>
+        </is>
+      </c>
+      <c r="E528" t="inlineStr"/>
+      <c r="F528" t="inlineStr">
+        <is>
+          <t>初めて</t>
+        </is>
+      </c>
+      <c r="G528" t="inlineStr">
+        <is>
+          <t>新宿からきました！</t>
+        </is>
+      </c>
+      <c r="H528" t="inlineStr"/>
+    </row>
+    <row r="529">
+      <c r="A529" t="n">
+        <v>27783</v>
+      </c>
+      <c r="B529" t="inlineStr">
+        <is>
+          <t>2026-09-15</t>
+        </is>
+      </c>
+      <c r="C529" t="inlineStr">
+        <is>
+          <t>02:46:10</t>
+        </is>
+      </c>
+      <c r="D529" t="inlineStr">
+        <is>
+          <t>ミカミと仲間たち</t>
+        </is>
+      </c>
+      <c r="E529" t="inlineStr"/>
+      <c r="F529" t="inlineStr">
+        <is>
+          <t>新規さん連れて</t>
+        </is>
+      </c>
+      <c r="G529" t="inlineStr">
+        <is>
+          <t>きたよー</t>
+        </is>
+      </c>
+      <c r="H529" t="inlineStr"/>
+    </row>
+    <row r="530">
+      <c r="A530" t="n">
+        <v>27785</v>
+      </c>
+      <c r="B530" t="inlineStr">
+        <is>
+          <t>2026-09-15</t>
+        </is>
+      </c>
+      <c r="C530" t="inlineStr">
+        <is>
+          <t>04:30:21</t>
+        </is>
+      </c>
+      <c r="D530" t="inlineStr">
+        <is>
+          <t>★BAMBITCH★</t>
+        </is>
+      </c>
+      <c r="E530" t="inlineStr">
+        <is>
+          <t>天然の100人ネキ　ねむ</t>
+        </is>
+      </c>
+      <c r="F530" t="inlineStr">
+        <is>
+          <t>★☆★朝までアゲアゲの火曜日営業が始まるわよ♪★☆★</t>
+        </is>
+      </c>
+      <c r="G530" t="inlineStr">
+        <is>
+          <t>本日9月15日の営業時間は♪
+オープン19:00！ラスト5:00なのよ☆
+担当は
+天然の100人ネキ　ねむ
+なのよ♪
+どんな季節でも★BAMBITCH★は色気ムンムンで暑すぎる♪
+バンビッチでおもいっきりはじけちゃって（笑）
+精力は無くても性欲がある！？
+大人の憩いと禁断サークル盛りだくさん！
+憩いと交流の魔性の遊び場バンビッチは素敵な出会いを 提供いたします（笑)☆☆
+おつまみ等の持ち込みは自由なのでみんなで持ち寄ってお近づきのきっかけにどうぞ♪
+強制や無理強いは一切ございませんので楽しく遊びましょう♪
+宇都宮市宿郷1−12−9　カサブランカビル5F</t>
+        </is>
+      </c>
+      <c r="H530" t="inlineStr">
+        <is>
+          <t>img20260915043021.jpg</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -16955,7 +17149,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I623"/>
+  <dimension ref="A1:I628"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -43758,6 +43952,221 @@
       <c r="I623" t="inlineStr">
         <is>
           <t>来たっちゃ</t>
+        </is>
+      </c>
+    </row>
+    <row r="624">
+      <c r="A624" t="inlineStr">
+        <is>
+          <t>2026-09-14</t>
+        </is>
+      </c>
+      <c r="B624" t="inlineStr">
+        <is>
+          <t>月</t>
+        </is>
+      </c>
+      <c r="C624" t="inlineStr">
+        <is>
+          <t>19:21:38</t>
+        </is>
+      </c>
+      <c r="D624" t="n">
+        <v>27775</v>
+      </c>
+      <c r="E624" t="inlineStr">
+        <is>
+          <t>ひがん</t>
+        </is>
+      </c>
+      <c r="F624" t="n">
+        <v>17</v>
+      </c>
+      <c r="G624" t="inlineStr">
+        <is>
+          <t>ひがん</t>
+        </is>
+      </c>
+      <c r="H624" t="inlineStr">
+        <is>
+          <t>ちいかわ観て</t>
+        </is>
+      </c>
+      <c r="I624" t="inlineStr">
+        <is>
+          <t>来ました♪</t>
+        </is>
+      </c>
+    </row>
+    <row r="625">
+      <c r="A625" t="inlineStr">
+        <is>
+          <t>2026-09-14</t>
+        </is>
+      </c>
+      <c r="B625" t="inlineStr">
+        <is>
+          <t>月</t>
+        </is>
+      </c>
+      <c r="C625" t="inlineStr">
+        <is>
+          <t>19:22:11</t>
+        </is>
+      </c>
+      <c r="D625" t="n">
+        <v>27776</v>
+      </c>
+      <c r="E625" t="inlineStr">
+        <is>
+          <t>bee</t>
+        </is>
+      </c>
+      <c r="F625" t="n">
+        <v>4</v>
+      </c>
+      <c r="G625" t="inlineStr">
+        <is>
+          <t>bee</t>
+        </is>
+      </c>
+      <c r="H625" t="inlineStr">
+        <is>
+          <t>遊びに</t>
+        </is>
+      </c>
+      <c r="I625" t="inlineStr">
+        <is>
+          <t>来ましたブン♪</t>
+        </is>
+      </c>
+    </row>
+    <row r="626">
+      <c r="A626" t="inlineStr">
+        <is>
+          <t>2026-09-14</t>
+        </is>
+      </c>
+      <c r="B626" t="inlineStr">
+        <is>
+          <t>月</t>
+        </is>
+      </c>
+      <c r="C626" t="inlineStr">
+        <is>
+          <t>19:57:51</t>
+        </is>
+      </c>
+      <c r="D626" t="n">
+        <v>27779</v>
+      </c>
+      <c r="E626" t="inlineStr">
+        <is>
+          <t>ろくじ</t>
+        </is>
+      </c>
+      <c r="F626" t="n">
+        <v>4</v>
+      </c>
+      <c r="G626" t="inlineStr">
+        <is>
+          <t>ろくじ</t>
+        </is>
+      </c>
+      <c r="H626" t="inlineStr">
+        <is>
+          <t>飲みに</t>
+        </is>
+      </c>
+      <c r="I626" t="inlineStr">
+        <is>
+          <t>来ました！</t>
+        </is>
+      </c>
+    </row>
+    <row r="627">
+      <c r="A627" t="inlineStr">
+        <is>
+          <t>2026-09-14</t>
+        </is>
+      </c>
+      <c r="B627" t="inlineStr">
+        <is>
+          <t>月</t>
+        </is>
+      </c>
+      <c r="C627" t="inlineStr">
+        <is>
+          <t>20:43:04</t>
+        </is>
+      </c>
+      <c r="D627" t="n">
+        <v>27780</v>
+      </c>
+      <c r="E627" t="inlineStr">
+        <is>
+          <t>まみ</t>
+        </is>
+      </c>
+      <c r="F627" t="n">
+        <v>1</v>
+      </c>
+      <c r="G627" t="inlineStr">
+        <is>
+          <t>まみ</t>
+        </is>
+      </c>
+      <c r="H627" t="inlineStr">
+        <is>
+          <t>初めて</t>
+        </is>
+      </c>
+      <c r="I627" t="inlineStr">
+        <is>
+          <t>新宿からきました！</t>
+        </is>
+      </c>
+    </row>
+    <row r="628">
+      <c r="A628" t="inlineStr">
+        <is>
+          <t>2026-09-15</t>
+        </is>
+      </c>
+      <c r="B628" t="inlineStr">
+        <is>
+          <t>火</t>
+        </is>
+      </c>
+      <c r="C628" t="inlineStr">
+        <is>
+          <t>02:46:10</t>
+        </is>
+      </c>
+      <c r="D628" t="n">
+        <v>27783</v>
+      </c>
+      <c r="E628" t="inlineStr">
+        <is>
+          <t>ミカミと仲間たち</t>
+        </is>
+      </c>
+      <c r="F628" t="n">
+        <v>1</v>
+      </c>
+      <c r="G628" t="inlineStr">
+        <is>
+          <t>ミカミと仲間たち</t>
+        </is>
+      </c>
+      <c r="H628" t="inlineStr">
+        <is>
+          <t>新規さん連れて</t>
+        </is>
+      </c>
+      <c r="I628" t="inlineStr">
+        <is>
+          <t>きたよー</t>
         </is>
       </c>
     </row>
@@ -43772,7 +44181,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D370"/>
+  <dimension ref="A1:D372"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -43804,7 +44213,7 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="C2" t="inlineStr">
         <is>
@@ -44220,7 +44629,7 @@
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>かず</t>
+          <t>bee</t>
         </is>
       </c>
       <c r="B23" t="n">
@@ -44228,19 +44637,19 @@
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>2026-08-16</t>
+          <t>2026-08-14</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>2026-09-12</t>
+          <t>2026-09-14</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>くれは</t>
+          <t>かず</t>
         </is>
       </c>
       <c r="B24" t="n">
@@ -44248,19 +44657,19 @@
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>2026-09-01</t>
+          <t>2026-08-16</t>
         </is>
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>2026-09-13</t>
+          <t>2026-09-12</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>すず</t>
+          <t>くれは</t>
         </is>
       </c>
       <c r="B25" t="n">
@@ -44268,19 +44677,19 @@
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>2026-08-16</t>
+          <t>2026-09-01</t>
         </is>
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>2026-09-06</t>
+          <t>2026-09-13</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>たかやま</t>
+          <t>すず</t>
         </is>
       </c>
       <c r="B26" t="n">
@@ -44288,19 +44697,19 @@
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>2026-08-13</t>
+          <t>2026-08-16</t>
         </is>
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>2026-09-08</t>
+          <t>2026-09-06</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>まいなちゅ</t>
+          <t>たかやま</t>
         </is>
       </c>
       <c r="B27" t="n">
@@ -44308,19 +44717,19 @@
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>2026-08-15</t>
+          <t>2026-08-13</t>
         </is>
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>2026-08-29</t>
+          <t>2026-09-08</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>まーくん</t>
+          <t>まいなちゅ</t>
         </is>
       </c>
       <c r="B28" t="n">
@@ -44328,19 +44737,19 @@
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>2026-08-16</t>
+          <t>2026-08-15</t>
         </is>
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>2026-09-07</t>
+          <t>2026-08-29</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>ゆう</t>
+          <t>まーくん</t>
         </is>
       </c>
       <c r="B29" t="n">
@@ -44348,19 +44757,19 @@
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>2026-08-20</t>
+          <t>2026-08-16</t>
         </is>
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>2026-09-13</t>
+          <t>2026-09-07</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>ゆうき</t>
+          <t>ゆう</t>
         </is>
       </c>
       <c r="B30" t="n">
@@ -44368,19 +44777,19 @@
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>2026-08-11</t>
+          <t>2026-08-20</t>
         </is>
       </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t>2026-09-05</t>
+          <t>2026-09-13</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>るい</t>
+          <t>ゆうき</t>
         </is>
       </c>
       <c r="B31" t="n">
@@ -44388,59 +44797,59 @@
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>2026-08-14</t>
+          <t>2026-08-11</t>
         </is>
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t>2026-09-10</t>
+          <t>2026-09-05</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>H</t>
+          <t>るい</t>
         </is>
       </c>
       <c r="B32" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>2026-08-11</t>
+          <t>2026-08-14</t>
         </is>
       </c>
       <c r="D32" t="inlineStr">
         <is>
-          <t>2026-09-02</t>
+          <t>2026-09-10</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>K</t>
+          <t>ろくじ</t>
         </is>
       </c>
       <c r="B33" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>2026-08-16</t>
+          <t>2026-08-19</t>
         </is>
       </c>
       <c r="D33" t="inlineStr">
         <is>
-          <t>2026-09-08</t>
+          <t>2026-09-14</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>S</t>
+          <t>H</t>
         </is>
       </c>
       <c r="B34" t="n">
@@ -44448,19 +44857,19 @@
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>2026-08-15</t>
+          <t>2026-08-11</t>
         </is>
       </c>
       <c r="D34" t="inlineStr">
         <is>
-          <t>2026-08-24</t>
+          <t>2026-09-02</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>T山</t>
+          <t>K</t>
         </is>
       </c>
       <c r="B35" t="n">
@@ -44468,19 +44877,19 @@
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>2026-08-10</t>
+          <t>2026-08-16</t>
         </is>
       </c>
       <c r="D35" t="inlineStr">
         <is>
-          <t>2026-08-30</t>
+          <t>2026-09-08</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>bee</t>
+          <t>S</t>
         </is>
       </c>
       <c r="B36" t="n">
@@ -44488,19 +44897,19 @@
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>2026-08-14</t>
+          <t>2026-08-15</t>
         </is>
       </c>
       <c r="D36" t="inlineStr">
         <is>
-          <t>2026-09-07</t>
+          <t>2026-08-24</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>あや</t>
+          <t>T山</t>
         </is>
       </c>
       <c r="B37" t="n">
@@ -44508,19 +44917,19 @@
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>2026-08-11</t>
+          <t>2026-08-10</t>
         </is>
       </c>
       <c r="D37" t="inlineStr">
         <is>
-          <t>2026-09-12</t>
+          <t>2026-08-30</t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>かな</t>
+          <t>あや</t>
         </is>
       </c>
       <c r="B38" t="n">
@@ -44528,19 +44937,19 @@
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>2026-08-12</t>
+          <t>2026-08-11</t>
         </is>
       </c>
       <c r="D38" t="inlineStr">
         <is>
-          <t>2026-08-30</t>
+          <t>2026-09-12</t>
         </is>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>こてっちゃん</t>
+          <t>かな</t>
         </is>
       </c>
       <c r="B39" t="n">
@@ -44548,19 +44957,19 @@
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>2026-08-15</t>
+          <t>2026-08-12</t>
         </is>
       </c>
       <c r="D39" t="inlineStr">
         <is>
-          <t>2026-09-08</t>
+          <t>2026-08-30</t>
         </is>
       </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>さと</t>
+          <t>こてっちゃん</t>
         </is>
       </c>
       <c r="B40" t="n">
@@ -44568,19 +44977,19 @@
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>2026-08-22</t>
+          <t>2026-08-15</t>
         </is>
       </c>
       <c r="D40" t="inlineStr">
         <is>
-          <t>2026-09-12</t>
+          <t>2026-09-08</t>
         </is>
       </c>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>すー</t>
+          <t>さと</t>
         </is>
       </c>
       <c r="B41" t="n">
@@ -44588,19 +44997,19 @@
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>2026-08-13</t>
+          <t>2026-08-22</t>
         </is>
       </c>
       <c r="D41" t="inlineStr">
         <is>
-          <t>2026-09-08</t>
+          <t>2026-09-12</t>
         </is>
       </c>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>すーさん</t>
+          <t>すー</t>
         </is>
       </c>
       <c r="B42" t="n">
@@ -44608,19 +45017,19 @@
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>2026-08-18</t>
+          <t>2026-08-13</t>
         </is>
       </c>
       <c r="D42" t="inlineStr">
         <is>
-          <t>2026-08-28</t>
+          <t>2026-09-08</t>
         </is>
       </c>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>だいご</t>
+          <t>すーさん</t>
         </is>
       </c>
       <c r="B43" t="n">
@@ -44628,19 +45037,19 @@
       </c>
       <c r="C43" t="inlineStr">
         <is>
-          <t>2026-08-15</t>
+          <t>2026-08-18</t>
         </is>
       </c>
       <c r="D43" t="inlineStr">
         <is>
-          <t>2026-09-12</t>
+          <t>2026-08-28</t>
         </is>
       </c>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>てくのちゃん</t>
+          <t>だいご</t>
         </is>
       </c>
       <c r="B44" t="n">
@@ -44648,19 +45057,19 @@
       </c>
       <c r="C44" t="inlineStr">
         <is>
-          <t>2026-08-27</t>
+          <t>2026-08-15</t>
         </is>
       </c>
       <c r="D44" t="inlineStr">
         <is>
-          <t>2026-08-30</t>
+          <t>2026-09-12</t>
         </is>
       </c>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>でで</t>
+          <t>てくのちゃん</t>
         </is>
       </c>
       <c r="B45" t="n">
@@ -44668,19 +45077,19 @@
       </c>
       <c r="C45" t="inlineStr">
         <is>
-          <t>2026-08-10</t>
+          <t>2026-08-27</t>
         </is>
       </c>
       <c r="D45" t="inlineStr">
         <is>
-          <t>2026-09-04</t>
+          <t>2026-08-30</t>
         </is>
       </c>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>ひがんたん</t>
+          <t>でで</t>
         </is>
       </c>
       <c r="B46" t="n">
@@ -44688,19 +45097,19 @@
       </c>
       <c r="C46" t="inlineStr">
         <is>
-          <t>2026-08-20</t>
+          <t>2026-08-10</t>
         </is>
       </c>
       <c r="D46" t="inlineStr">
         <is>
-          <t>2026-09-07</t>
+          <t>2026-09-04</t>
         </is>
       </c>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>ゆずきん</t>
+          <t>ひがんたん</t>
         </is>
       </c>
       <c r="B47" t="n">
@@ -44713,14 +45122,14 @@
       </c>
       <c r="D47" t="inlineStr">
         <is>
-          <t>2026-08-26</t>
+          <t>2026-09-07</t>
         </is>
       </c>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>よしお</t>
+          <t>ゆずきん</t>
         </is>
       </c>
       <c r="B48" t="n">
@@ -44728,19 +45137,19 @@
       </c>
       <c r="C48" t="inlineStr">
         <is>
-          <t>2026-08-18</t>
+          <t>2026-08-20</t>
         </is>
       </c>
       <c r="D48" t="inlineStr">
         <is>
-          <t>2026-09-07</t>
+          <t>2026-08-26</t>
         </is>
       </c>
     </row>
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>よしおたん</t>
+          <t>よしお</t>
         </is>
       </c>
       <c r="B49" t="n">
@@ -44748,19 +45157,19 @@
       </c>
       <c r="C49" t="inlineStr">
         <is>
-          <t>2026-08-12</t>
+          <t>2026-08-18</t>
         </is>
       </c>
       <c r="D49" t="inlineStr">
         <is>
-          <t>2026-08-23</t>
+          <t>2026-09-07</t>
         </is>
       </c>
     </row>
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>れいら</t>
+          <t>よしおたん</t>
         </is>
       </c>
       <c r="B50" t="n">
@@ -44768,19 +45177,19 @@
       </c>
       <c r="C50" t="inlineStr">
         <is>
-          <t>2026-08-17</t>
+          <t>2026-08-12</t>
         </is>
       </c>
       <c r="D50" t="inlineStr">
         <is>
-          <t>2026-09-10</t>
+          <t>2026-08-23</t>
         </is>
       </c>
     </row>
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>ろくじ</t>
+          <t>れいら</t>
         </is>
       </c>
       <c r="B51" t="n">
@@ -44788,12 +45197,12 @@
       </c>
       <c r="C51" t="inlineStr">
         <is>
-          <t>2026-08-19</t>
+          <t>2026-08-17</t>
         </is>
       </c>
       <c r="D51" t="inlineStr">
         <is>
-          <t>2026-09-09</t>
+          <t>2026-09-10</t>
         </is>
       </c>
     </row>
@@ -48540,7 +48949,7 @@
     <row r="239">
       <c r="A239" t="inlineStr">
         <is>
-          <t>まや</t>
+          <t>まみ</t>
         </is>
       </c>
       <c r="B239" t="n">
@@ -48548,19 +48957,19 @@
       </c>
       <c r="C239" t="inlineStr">
         <is>
-          <t>2026-08-29</t>
+          <t>2026-09-14</t>
         </is>
       </c>
       <c r="D239" t="inlineStr">
         <is>
-          <t>2026-08-29</t>
+          <t>2026-09-14</t>
         </is>
       </c>
     </row>
     <row r="240">
       <c r="A240" t="inlineStr">
         <is>
-          <t>まり</t>
+          <t>まや</t>
         </is>
       </c>
       <c r="B240" t="n">
@@ -48568,19 +48977,19 @@
       </c>
       <c r="C240" t="inlineStr">
         <is>
-          <t>2026-09-13</t>
+          <t>2026-08-29</t>
         </is>
       </c>
       <c r="D240" t="inlineStr">
         <is>
-          <t>2026-09-13</t>
+          <t>2026-08-29</t>
         </is>
       </c>
     </row>
     <row r="241">
       <c r="A241" t="inlineStr">
         <is>
-          <t>まりん</t>
+          <t>まり</t>
         </is>
       </c>
       <c r="B241" t="n">
@@ -48588,19 +48997,19 @@
       </c>
       <c r="C241" t="inlineStr">
         <is>
-          <t>2026-08-15</t>
+          <t>2026-09-13</t>
         </is>
       </c>
       <c r="D241" t="inlineStr">
         <is>
-          <t>2026-08-15</t>
+          <t>2026-09-13</t>
         </is>
       </c>
     </row>
     <row r="242">
       <c r="A242" t="inlineStr">
         <is>
-          <t>まー</t>
+          <t>まりん</t>
         </is>
       </c>
       <c r="B242" t="n">
@@ -48608,19 +49017,19 @@
       </c>
       <c r="C242" t="inlineStr">
         <is>
-          <t>2026-08-30</t>
+          <t>2026-08-15</t>
         </is>
       </c>
       <c r="D242" t="inlineStr">
         <is>
-          <t>2026-08-30</t>
+          <t>2026-08-15</t>
         </is>
       </c>
     </row>
     <row r="243">
       <c r="A243" t="inlineStr">
         <is>
-          <t>まーさん</t>
+          <t>まー</t>
         </is>
       </c>
       <c r="B243" t="n">
@@ -48628,19 +49037,19 @@
       </c>
       <c r="C243" t="inlineStr">
         <is>
-          <t>2026-08-23</t>
+          <t>2026-08-30</t>
         </is>
       </c>
       <c r="D243" t="inlineStr">
         <is>
-          <t>2026-08-23</t>
+          <t>2026-08-30</t>
         </is>
       </c>
     </row>
     <row r="244">
       <c r="A244" t="inlineStr">
         <is>
-          <t>まーちゃん</t>
+          <t>まーさん</t>
         </is>
       </c>
       <c r="B244" t="n">
@@ -48648,19 +49057,19 @@
       </c>
       <c r="C244" t="inlineStr">
         <is>
-          <t>2026-09-07</t>
+          <t>2026-08-23</t>
         </is>
       </c>
       <c r="D244" t="inlineStr">
         <is>
-          <t>2026-09-07</t>
+          <t>2026-08-23</t>
         </is>
       </c>
     </row>
     <row r="245">
       <c r="A245" t="inlineStr">
         <is>
-          <t>みかん</t>
+          <t>まーちゃん</t>
         </is>
       </c>
       <c r="B245" t="n">
@@ -48668,19 +49077,19 @@
       </c>
       <c r="C245" t="inlineStr">
         <is>
-          <t>2026-08-16</t>
+          <t>2026-09-07</t>
         </is>
       </c>
       <c r="D245" t="inlineStr">
         <is>
-          <t>2026-08-16</t>
+          <t>2026-09-07</t>
         </is>
       </c>
     </row>
     <row r="246">
       <c r="A246" t="inlineStr">
         <is>
-          <t>みずき</t>
+          <t>みかん</t>
         </is>
       </c>
       <c r="B246" t="n">
@@ -48700,7 +49109,7 @@
     <row r="247">
       <c r="A247" t="inlineStr">
         <is>
-          <t>みちゃ</t>
+          <t>みずき</t>
         </is>
       </c>
       <c r="B247" t="n">
@@ -48708,19 +49117,19 @@
       </c>
       <c r="C247" t="inlineStr">
         <is>
-          <t>2026-08-20</t>
+          <t>2026-08-16</t>
         </is>
       </c>
       <c r="D247" t="inlineStr">
         <is>
-          <t>2026-08-20</t>
+          <t>2026-08-16</t>
         </is>
       </c>
     </row>
     <row r="248">
       <c r="A248" t="inlineStr">
         <is>
-          <t>みっちー</t>
+          <t>みちゃ</t>
         </is>
       </c>
       <c r="B248" t="n">
@@ -48728,19 +49137,19 @@
       </c>
       <c r="C248" t="inlineStr">
         <is>
-          <t>2026-09-04</t>
+          <t>2026-08-20</t>
         </is>
       </c>
       <c r="D248" t="inlineStr">
         <is>
-          <t>2026-09-04</t>
+          <t>2026-08-20</t>
         </is>
       </c>
     </row>
     <row r="249">
       <c r="A249" t="inlineStr">
         <is>
-          <t>みなつちん</t>
+          <t>みっちー</t>
         </is>
       </c>
       <c r="B249" t="n">
@@ -48748,19 +49157,19 @@
       </c>
       <c r="C249" t="inlineStr">
         <is>
-          <t>2026-08-16</t>
+          <t>2026-09-04</t>
         </is>
       </c>
       <c r="D249" t="inlineStr">
         <is>
-          <t>2026-08-16</t>
+          <t>2026-09-04</t>
         </is>
       </c>
     </row>
     <row r="250">
       <c r="A250" t="inlineStr">
         <is>
-          <t>みみ</t>
+          <t>みなつちん</t>
         </is>
       </c>
       <c r="B250" t="n">
@@ -48768,19 +49177,19 @@
       </c>
       <c r="C250" t="inlineStr">
         <is>
-          <t>2026-08-26</t>
+          <t>2026-08-16</t>
         </is>
       </c>
       <c r="D250" t="inlineStr">
         <is>
-          <t>2026-08-26</t>
+          <t>2026-08-16</t>
         </is>
       </c>
     </row>
     <row r="251">
       <c r="A251" t="inlineStr">
         <is>
-          <t>みゆき</t>
+          <t>みみ</t>
         </is>
       </c>
       <c r="B251" t="n">
@@ -48788,19 +49197,19 @@
       </c>
       <c r="C251" t="inlineStr">
         <is>
-          <t>2026-09-05</t>
+          <t>2026-08-26</t>
         </is>
       </c>
       <c r="D251" t="inlineStr">
         <is>
-          <t>2026-09-05</t>
+          <t>2026-08-26</t>
         </is>
       </c>
     </row>
     <row r="252">
       <c r="A252" t="inlineStr">
         <is>
-          <t>みらい</t>
+          <t>みゆき</t>
         </is>
       </c>
       <c r="B252" t="n">
@@ -48808,19 +49217,19 @@
       </c>
       <c r="C252" t="inlineStr">
         <is>
-          <t>2026-08-29</t>
+          <t>2026-09-05</t>
         </is>
       </c>
       <c r="D252" t="inlineStr">
         <is>
-          <t>2026-08-29</t>
+          <t>2026-09-05</t>
         </is>
       </c>
     </row>
     <row r="253">
       <c r="A253" t="inlineStr">
         <is>
-          <t>みるこ</t>
+          <t>みらい</t>
         </is>
       </c>
       <c r="B253" t="n">
@@ -48828,19 +49237,19 @@
       </c>
       <c r="C253" t="inlineStr">
         <is>
-          <t>2026-08-19</t>
+          <t>2026-08-29</t>
         </is>
       </c>
       <c r="D253" t="inlineStr">
         <is>
-          <t>2026-08-19</t>
+          <t>2026-08-29</t>
         </is>
       </c>
     </row>
     <row r="254">
       <c r="A254" t="inlineStr">
         <is>
-          <t>みん</t>
+          <t>みるこ</t>
         </is>
       </c>
       <c r="B254" t="n">
@@ -48848,19 +49257,19 @@
       </c>
       <c r="C254" t="inlineStr">
         <is>
-          <t>2026-09-12</t>
+          <t>2026-08-19</t>
         </is>
       </c>
       <c r="D254" t="inlineStr">
         <is>
-          <t>2026-09-12</t>
+          <t>2026-08-19</t>
         </is>
       </c>
     </row>
     <row r="255">
       <c r="A255" t="inlineStr">
         <is>
-          <t>みー</t>
+          <t>みん</t>
         </is>
       </c>
       <c r="B255" t="n">
@@ -48868,19 +49277,19 @@
       </c>
       <c r="C255" t="inlineStr">
         <is>
-          <t>2026-09-13</t>
+          <t>2026-09-12</t>
         </is>
       </c>
       <c r="D255" t="inlineStr">
         <is>
-          <t>2026-09-13</t>
+          <t>2026-09-12</t>
         </is>
       </c>
     </row>
     <row r="256">
       <c r="A256" t="inlineStr">
         <is>
-          <t>みーみ</t>
+          <t>みー</t>
         </is>
       </c>
       <c r="B256" t="n">
@@ -48888,19 +49297,19 @@
       </c>
       <c r="C256" t="inlineStr">
         <is>
-          <t>2026-08-15</t>
+          <t>2026-09-13</t>
         </is>
       </c>
       <c r="D256" t="inlineStr">
         <is>
-          <t>2026-08-15</t>
+          <t>2026-09-13</t>
         </is>
       </c>
     </row>
     <row r="257">
       <c r="A257" t="inlineStr">
         <is>
-          <t>もかちんぽぽ</t>
+          <t>みーみ</t>
         </is>
       </c>
       <c r="B257" t="n">
@@ -48908,19 +49317,19 @@
       </c>
       <c r="C257" t="inlineStr">
         <is>
-          <t>2026-08-20</t>
+          <t>2026-08-15</t>
         </is>
       </c>
       <c r="D257" t="inlineStr">
         <is>
-          <t>2026-08-20</t>
+          <t>2026-08-15</t>
         </is>
       </c>
     </row>
     <row r="258">
       <c r="A258" t="inlineStr">
         <is>
-          <t>もっち</t>
+          <t>もかちんぽぽ</t>
         </is>
       </c>
       <c r="B258" t="n">
@@ -48928,19 +49337,19 @@
       </c>
       <c r="C258" t="inlineStr">
         <is>
-          <t>2026-09-04</t>
+          <t>2026-08-20</t>
         </is>
       </c>
       <c r="D258" t="inlineStr">
         <is>
-          <t>2026-09-04</t>
+          <t>2026-08-20</t>
         </is>
       </c>
     </row>
     <row r="259">
       <c r="A259" t="inlineStr">
         <is>
-          <t>もと</t>
+          <t>もっち</t>
         </is>
       </c>
       <c r="B259" t="n">
@@ -48948,19 +49357,19 @@
       </c>
       <c r="C259" t="inlineStr">
         <is>
-          <t>2026-09-03</t>
+          <t>2026-09-04</t>
         </is>
       </c>
       <c r="D259" t="inlineStr">
         <is>
-          <t>2026-09-03</t>
+          <t>2026-09-04</t>
         </is>
       </c>
     </row>
     <row r="260">
       <c r="A260" t="inlineStr">
         <is>
-          <t>ももたろ</t>
+          <t>もと</t>
         </is>
       </c>
       <c r="B260" t="n">
@@ -48968,19 +49377,19 @@
       </c>
       <c r="C260" t="inlineStr">
         <is>
-          <t>2026-08-10</t>
+          <t>2026-09-03</t>
         </is>
       </c>
       <c r="D260" t="inlineStr">
         <is>
-          <t>2026-08-10</t>
+          <t>2026-09-03</t>
         </is>
       </c>
     </row>
     <row r="261">
       <c r="A261" t="inlineStr">
         <is>
-          <t>ゆい</t>
+          <t>ももたろ</t>
         </is>
       </c>
       <c r="B261" t="n">
@@ -48988,19 +49397,19 @@
       </c>
       <c r="C261" t="inlineStr">
         <is>
-          <t>2026-09-04</t>
+          <t>2026-08-10</t>
         </is>
       </c>
       <c r="D261" t="inlineStr">
         <is>
-          <t>2026-09-04</t>
+          <t>2026-08-10</t>
         </is>
       </c>
     </row>
     <row r="262">
       <c r="A262" t="inlineStr">
         <is>
-          <t>ゆうくん</t>
+          <t>ゆい</t>
         </is>
       </c>
       <c r="B262" t="n">
@@ -49008,19 +49417,19 @@
       </c>
       <c r="C262" t="inlineStr">
         <is>
-          <t>2026-08-17</t>
+          <t>2026-09-04</t>
         </is>
       </c>
       <c r="D262" t="inlineStr">
         <is>
-          <t>2026-08-17</t>
+          <t>2026-09-04</t>
         </is>
       </c>
     </row>
     <row r="263">
       <c r="A263" t="inlineStr">
         <is>
-          <t>ゆうた</t>
+          <t>ゆうくん</t>
         </is>
       </c>
       <c r="B263" t="n">
@@ -49028,19 +49437,19 @@
       </c>
       <c r="C263" t="inlineStr">
         <is>
-          <t>2026-09-12</t>
+          <t>2026-08-17</t>
         </is>
       </c>
       <c r="D263" t="inlineStr">
         <is>
-          <t>2026-09-12</t>
+          <t>2026-08-17</t>
         </is>
       </c>
     </row>
     <row r="264">
       <c r="A264" t="inlineStr">
         <is>
-          <t>ゆうたん</t>
+          <t>ゆうた</t>
         </is>
       </c>
       <c r="B264" t="n">
@@ -49048,19 +49457,19 @@
       </c>
       <c r="C264" t="inlineStr">
         <is>
-          <t>2026-08-10</t>
+          <t>2026-09-12</t>
         </is>
       </c>
       <c r="D264" t="inlineStr">
         <is>
-          <t>2026-08-10</t>
+          <t>2026-09-12</t>
         </is>
       </c>
     </row>
     <row r="265">
       <c r="A265" t="inlineStr">
         <is>
-          <t>ゆうと</t>
+          <t>ゆうたん</t>
         </is>
       </c>
       <c r="B265" t="n">
@@ -49068,19 +49477,19 @@
       </c>
       <c r="C265" t="inlineStr">
         <is>
-          <t>2026-08-09</t>
+          <t>2026-08-10</t>
         </is>
       </c>
       <c r="D265" t="inlineStr">
         <is>
-          <t>2026-08-09</t>
+          <t>2026-08-10</t>
         </is>
       </c>
     </row>
     <row r="266">
       <c r="A266" t="inlineStr">
         <is>
-          <t>ゆうや</t>
+          <t>ゆうと</t>
         </is>
       </c>
       <c r="B266" t="n">
@@ -49088,19 +49497,19 @@
       </c>
       <c r="C266" t="inlineStr">
         <is>
-          <t>2026-08-20</t>
+          <t>2026-08-09</t>
         </is>
       </c>
       <c r="D266" t="inlineStr">
         <is>
-          <t>2026-08-20</t>
+          <t>2026-08-09</t>
         </is>
       </c>
     </row>
     <row r="267">
       <c r="A267" t="inlineStr">
         <is>
-          <t>ゆきんこ</t>
+          <t>ゆうや</t>
         </is>
       </c>
       <c r="B267" t="n">
@@ -49108,19 +49517,19 @@
       </c>
       <c r="C267" t="inlineStr">
         <is>
-          <t>2026-08-17</t>
+          <t>2026-08-20</t>
         </is>
       </c>
       <c r="D267" t="inlineStr">
         <is>
-          <t>2026-08-17</t>
+          <t>2026-08-20</t>
         </is>
       </c>
     </row>
     <row r="268">
       <c r="A268" t="inlineStr">
         <is>
-          <t>ゆず</t>
+          <t>ゆきんこ</t>
         </is>
       </c>
       <c r="B268" t="n">
@@ -49128,19 +49537,19 @@
       </c>
       <c r="C268" t="inlineStr">
         <is>
-          <t>2026-08-14</t>
+          <t>2026-08-17</t>
         </is>
       </c>
       <c r="D268" t="inlineStr">
         <is>
-          <t>2026-08-14</t>
+          <t>2026-08-17</t>
         </is>
       </c>
     </row>
     <row r="269">
       <c r="A269" t="inlineStr">
         <is>
-          <t>ゆずき＆ましゅ</t>
+          <t>ゆず</t>
         </is>
       </c>
       <c r="B269" t="n">
@@ -49148,19 +49557,19 @@
       </c>
       <c r="C269" t="inlineStr">
         <is>
-          <t>2026-08-30</t>
+          <t>2026-08-14</t>
         </is>
       </c>
       <c r="D269" t="inlineStr">
         <is>
-          <t>2026-08-30</t>
+          <t>2026-08-14</t>
         </is>
       </c>
     </row>
     <row r="270">
       <c r="A270" t="inlineStr">
         <is>
-          <t>ゆぴ</t>
+          <t>ゆずき＆ましゅ</t>
         </is>
       </c>
       <c r="B270" t="n">
@@ -49168,19 +49577,19 @@
       </c>
       <c r="C270" t="inlineStr">
         <is>
-          <t>2026-08-12</t>
+          <t>2026-08-30</t>
         </is>
       </c>
       <c r="D270" t="inlineStr">
         <is>
-          <t>2026-08-12</t>
+          <t>2026-08-30</t>
         </is>
       </c>
     </row>
     <row r="271">
       <c r="A271" t="inlineStr">
         <is>
-          <t>ゆり</t>
+          <t>ゆぴ</t>
         </is>
       </c>
       <c r="B271" t="n">
@@ -49188,19 +49597,19 @@
       </c>
       <c r="C271" t="inlineStr">
         <is>
-          <t>2026-08-14</t>
+          <t>2026-08-12</t>
         </is>
       </c>
       <c r="D271" t="inlineStr">
         <is>
-          <t>2026-08-14</t>
+          <t>2026-08-12</t>
         </is>
       </c>
     </row>
     <row r="272">
       <c r="A272" t="inlineStr">
         <is>
-          <t>ゆりな</t>
+          <t>ゆり</t>
         </is>
       </c>
       <c r="B272" t="n">
@@ -49208,19 +49617,19 @@
       </c>
       <c r="C272" t="inlineStr">
         <is>
-          <t>2026-09-05</t>
+          <t>2026-08-14</t>
         </is>
       </c>
       <c r="D272" t="inlineStr">
         <is>
-          <t>2026-09-05</t>
+          <t>2026-08-14</t>
         </is>
       </c>
     </row>
     <row r="273">
       <c r="A273" t="inlineStr">
         <is>
-          <t>ゆん</t>
+          <t>ゆりな</t>
         </is>
       </c>
       <c r="B273" t="n">
@@ -49228,19 +49637,19 @@
       </c>
       <c r="C273" t="inlineStr">
         <is>
-          <t>2026-08-10</t>
+          <t>2026-09-05</t>
         </is>
       </c>
       <c r="D273" t="inlineStr">
         <is>
-          <t>2026-08-10</t>
+          <t>2026-09-05</t>
         </is>
       </c>
     </row>
     <row r="274">
       <c r="A274" t="inlineStr">
         <is>
-          <t>よこい</t>
+          <t>ゆん</t>
         </is>
       </c>
       <c r="B274" t="n">
@@ -49248,19 +49657,19 @@
       </c>
       <c r="C274" t="inlineStr">
         <is>
-          <t>2026-09-01</t>
+          <t>2026-08-10</t>
         </is>
       </c>
       <c r="D274" t="inlineStr">
         <is>
-          <t>2026-09-01</t>
+          <t>2026-08-10</t>
         </is>
       </c>
     </row>
     <row r="275">
       <c r="A275" t="inlineStr">
         <is>
-          <t>よちお</t>
+          <t>よこい</t>
         </is>
       </c>
       <c r="B275" t="n">
@@ -49268,19 +49677,19 @@
       </c>
       <c r="C275" t="inlineStr">
         <is>
-          <t>2026-08-31</t>
+          <t>2026-09-01</t>
         </is>
       </c>
       <c r="D275" t="inlineStr">
         <is>
-          <t>2026-08-31</t>
+          <t>2026-09-01</t>
         </is>
       </c>
     </row>
     <row r="276">
       <c r="A276" t="inlineStr">
         <is>
-          <t>らうら</t>
+          <t>よちお</t>
         </is>
       </c>
       <c r="B276" t="n">
@@ -49288,19 +49697,19 @@
       </c>
       <c r="C276" t="inlineStr">
         <is>
-          <t>2026-08-10</t>
+          <t>2026-08-31</t>
         </is>
       </c>
       <c r="D276" t="inlineStr">
         <is>
-          <t>2026-08-10</t>
+          <t>2026-08-31</t>
         </is>
       </c>
     </row>
     <row r="277">
       <c r="A277" t="inlineStr">
         <is>
-          <t>らお</t>
+          <t>らうら</t>
         </is>
       </c>
       <c r="B277" t="n">
@@ -49308,19 +49717,19 @@
       </c>
       <c r="C277" t="inlineStr">
         <is>
-          <t>2026-08-26</t>
+          <t>2026-08-10</t>
         </is>
       </c>
       <c r="D277" t="inlineStr">
         <is>
-          <t>2026-08-26</t>
+          <t>2026-08-10</t>
         </is>
       </c>
     </row>
     <row r="278">
       <c r="A278" t="inlineStr">
         <is>
-          <t>りえ</t>
+          <t>らお</t>
         </is>
       </c>
       <c r="B278" t="n">
@@ -49328,19 +49737,19 @@
       </c>
       <c r="C278" t="inlineStr">
         <is>
-          <t>2026-08-14</t>
+          <t>2026-08-26</t>
         </is>
       </c>
       <c r="D278" t="inlineStr">
         <is>
-          <t>2026-08-14</t>
+          <t>2026-08-26</t>
         </is>
       </c>
     </row>
     <row r="279">
       <c r="A279" t="inlineStr">
         <is>
-          <t>りく</t>
+          <t>りえ</t>
         </is>
       </c>
       <c r="B279" t="n">
@@ -49348,19 +49757,19 @@
       </c>
       <c r="C279" t="inlineStr">
         <is>
-          <t>2026-08-16</t>
+          <t>2026-08-14</t>
         </is>
       </c>
       <c r="D279" t="inlineStr">
         <is>
-          <t>2026-08-16</t>
+          <t>2026-08-14</t>
         </is>
       </c>
     </row>
     <row r="280">
       <c r="A280" t="inlineStr">
         <is>
-          <t>りさ</t>
+          <t>りく</t>
         </is>
       </c>
       <c r="B280" t="n">
@@ -49368,19 +49777,19 @@
       </c>
       <c r="C280" t="inlineStr">
         <is>
-          <t>2026-08-13</t>
+          <t>2026-08-16</t>
         </is>
       </c>
       <c r="D280" t="inlineStr">
         <is>
-          <t>2026-08-13</t>
+          <t>2026-08-16</t>
         </is>
       </c>
     </row>
     <row r="281">
       <c r="A281" t="inlineStr">
         <is>
-          <t>りゅうくん</t>
+          <t>りさ</t>
         </is>
       </c>
       <c r="B281" t="n">
@@ -49388,19 +49797,19 @@
       </c>
       <c r="C281" t="inlineStr">
         <is>
-          <t>2026-08-22</t>
+          <t>2026-08-13</t>
         </is>
       </c>
       <c r="D281" t="inlineStr">
         <is>
-          <t>2026-08-22</t>
+          <t>2026-08-13</t>
         </is>
       </c>
     </row>
     <row r="282">
       <c r="A282" t="inlineStr">
         <is>
-          <t>りゅーちゃん</t>
+          <t>りゅうくん</t>
         </is>
       </c>
       <c r="B282" t="n">
@@ -49408,19 +49817,19 @@
       </c>
       <c r="C282" t="inlineStr">
         <is>
-          <t>2026-09-13</t>
+          <t>2026-08-22</t>
         </is>
       </c>
       <c r="D282" t="inlineStr">
         <is>
-          <t>2026-09-13</t>
+          <t>2026-08-22</t>
         </is>
       </c>
     </row>
     <row r="283">
       <c r="A283" t="inlineStr">
         <is>
-          <t>りょうが</t>
+          <t>りゅーちゃん</t>
         </is>
       </c>
       <c r="B283" t="n">
@@ -49440,7 +49849,7 @@
     <row r="284">
       <c r="A284" t="inlineStr">
         <is>
-          <t>りょうちゃん</t>
+          <t>りょうが</t>
         </is>
       </c>
       <c r="B284" t="n">
@@ -49448,19 +49857,19 @@
       </c>
       <c r="C284" t="inlineStr">
         <is>
-          <t>2026-08-10</t>
+          <t>2026-09-13</t>
         </is>
       </c>
       <c r="D284" t="inlineStr">
         <is>
-          <t>2026-08-10</t>
+          <t>2026-09-13</t>
         </is>
       </c>
     </row>
     <row r="285">
       <c r="A285" t="inlineStr">
         <is>
-          <t>りょーが</t>
+          <t>りょうちゃん</t>
         </is>
       </c>
       <c r="B285" t="n">
@@ -49468,19 +49877,19 @@
       </c>
       <c r="C285" t="inlineStr">
         <is>
-          <t>2026-09-06</t>
+          <t>2026-08-10</t>
         </is>
       </c>
       <c r="D285" t="inlineStr">
         <is>
-          <t>2026-09-06</t>
+          <t>2026-08-10</t>
         </is>
       </c>
     </row>
     <row r="286">
       <c r="A286" t="inlineStr">
         <is>
-          <t>りりこ</t>
+          <t>りょーが</t>
         </is>
       </c>
       <c r="B286" t="n">
@@ -49488,19 +49897,19 @@
       </c>
       <c r="C286" t="inlineStr">
         <is>
-          <t>2026-08-13</t>
+          <t>2026-09-06</t>
         </is>
       </c>
       <c r="D286" t="inlineStr">
         <is>
-          <t>2026-08-13</t>
+          <t>2026-09-06</t>
         </is>
       </c>
     </row>
     <row r="287">
       <c r="A287" t="inlineStr">
         <is>
-          <t>りん＆ゆち</t>
+          <t>りりこ</t>
         </is>
       </c>
       <c r="B287" t="n">
@@ -49508,19 +49917,19 @@
       </c>
       <c r="C287" t="inlineStr">
         <is>
-          <t>2026-08-28</t>
+          <t>2026-08-13</t>
         </is>
       </c>
       <c r="D287" t="inlineStr">
         <is>
-          <t>2026-08-28</t>
+          <t>2026-08-13</t>
         </is>
       </c>
     </row>
     <row r="288">
       <c r="A288" t="inlineStr">
         <is>
-          <t>れー</t>
+          <t>りん＆ゆち</t>
         </is>
       </c>
       <c r="B288" t="n">
@@ -49528,19 +49937,19 @@
       </c>
       <c r="C288" t="inlineStr">
         <is>
-          <t>2026-08-16</t>
+          <t>2026-08-28</t>
         </is>
       </c>
       <c r="D288" t="inlineStr">
         <is>
-          <t>2026-08-16</t>
+          <t>2026-08-28</t>
         </is>
       </c>
     </row>
     <row r="289">
       <c r="A289" t="inlineStr">
         <is>
-          <t>アイ</t>
+          <t>れー</t>
         </is>
       </c>
       <c r="B289" t="n">
@@ -49548,19 +49957,19 @@
       </c>
       <c r="C289" t="inlineStr">
         <is>
-          <t>2026-09-03</t>
+          <t>2026-08-16</t>
         </is>
       </c>
       <c r="D289" t="inlineStr">
         <is>
-          <t>2026-09-03</t>
+          <t>2026-08-16</t>
         </is>
       </c>
     </row>
     <row r="290">
       <c r="A290" t="inlineStr">
         <is>
-          <t>アイちゃん</t>
+          <t>アイ</t>
         </is>
       </c>
       <c r="B290" t="n">
@@ -49568,19 +49977,19 @@
       </c>
       <c r="C290" t="inlineStr">
         <is>
-          <t>2026-08-28</t>
+          <t>2026-09-03</t>
         </is>
       </c>
       <c r="D290" t="inlineStr">
         <is>
-          <t>2026-08-28</t>
+          <t>2026-09-03</t>
         </is>
       </c>
     </row>
     <row r="291">
       <c r="A291" t="inlineStr">
         <is>
-          <t>アキ</t>
+          <t>アイちゃん</t>
         </is>
       </c>
       <c r="B291" t="n">
@@ -49588,19 +49997,19 @@
       </c>
       <c r="C291" t="inlineStr">
         <is>
-          <t>2026-08-11</t>
+          <t>2026-08-28</t>
         </is>
       </c>
       <c r="D291" t="inlineStr">
         <is>
-          <t>2026-08-11</t>
+          <t>2026-08-28</t>
         </is>
       </c>
     </row>
     <row r="292">
       <c r="A292" t="inlineStr">
         <is>
-          <t>アナルプリンス</t>
+          <t>アキ</t>
         </is>
       </c>
       <c r="B292" t="n">
@@ -49608,19 +50017,19 @@
       </c>
       <c r="C292" t="inlineStr">
         <is>
-          <t>2026-08-22</t>
+          <t>2026-08-11</t>
         </is>
       </c>
       <c r="D292" t="inlineStr">
         <is>
-          <t>2026-08-22</t>
+          <t>2026-08-11</t>
         </is>
       </c>
     </row>
     <row r="293">
       <c r="A293" t="inlineStr">
         <is>
-          <t>イエモン</t>
+          <t>アナルプリンス</t>
         </is>
       </c>
       <c r="B293" t="n">
@@ -49628,19 +50037,19 @@
       </c>
       <c r="C293" t="inlineStr">
         <is>
-          <t>2026-09-03</t>
+          <t>2026-08-22</t>
         </is>
       </c>
       <c r="D293" t="inlineStr">
         <is>
-          <t>2026-09-03</t>
+          <t>2026-08-22</t>
         </is>
       </c>
     </row>
     <row r="294">
       <c r="A294" t="inlineStr">
         <is>
-          <t>オ・スー</t>
+          <t>イエモン</t>
         </is>
       </c>
       <c r="B294" t="n">
@@ -49648,19 +50057,19 @@
       </c>
       <c r="C294" t="inlineStr">
         <is>
-          <t>2026-08-13</t>
+          <t>2026-09-03</t>
         </is>
       </c>
       <c r="D294" t="inlineStr">
         <is>
-          <t>2026-08-13</t>
+          <t>2026-09-03</t>
         </is>
       </c>
     </row>
     <row r="295">
       <c r="A295" t="inlineStr">
         <is>
-          <t>カイト</t>
+          <t>オ・スー</t>
         </is>
       </c>
       <c r="B295" t="n">
@@ -49668,19 +50077,19 @@
       </c>
       <c r="C295" t="inlineStr">
         <is>
-          <t>2026-09-05</t>
+          <t>2026-08-13</t>
         </is>
       </c>
       <c r="D295" t="inlineStr">
         <is>
-          <t>2026-09-05</t>
+          <t>2026-08-13</t>
         </is>
       </c>
     </row>
     <row r="296">
       <c r="A296" t="inlineStr">
         <is>
-          <t>カズヤ</t>
+          <t>カイト</t>
         </is>
       </c>
       <c r="B296" t="n">
@@ -49700,7 +50109,7 @@
     <row r="297">
       <c r="A297" t="inlineStr">
         <is>
-          <t>カミさん</t>
+          <t>カズヤ</t>
         </is>
       </c>
       <c r="B297" t="n">
@@ -49708,19 +50117,19 @@
       </c>
       <c r="C297" t="inlineStr">
         <is>
-          <t>2026-08-22</t>
+          <t>2026-09-05</t>
         </is>
       </c>
       <c r="D297" t="inlineStr">
         <is>
-          <t>2026-08-22</t>
+          <t>2026-09-05</t>
         </is>
       </c>
     </row>
     <row r="298">
       <c r="A298" t="inlineStr">
         <is>
-          <t>カモリ</t>
+          <t>カミさん</t>
         </is>
       </c>
       <c r="B298" t="n">
@@ -49728,19 +50137,19 @@
       </c>
       <c r="C298" t="inlineStr">
         <is>
-          <t>2026-08-10</t>
+          <t>2026-08-22</t>
         </is>
       </c>
       <c r="D298" t="inlineStr">
         <is>
-          <t>2026-08-10</t>
+          <t>2026-08-22</t>
         </is>
       </c>
     </row>
     <row r="299">
       <c r="A299" t="inlineStr">
         <is>
-          <t>カー</t>
+          <t>カモリ</t>
         </is>
       </c>
       <c r="B299" t="n">
@@ -49748,19 +50157,19 @@
       </c>
       <c r="C299" t="inlineStr">
         <is>
-          <t>2026-08-09</t>
+          <t>2026-08-10</t>
         </is>
       </c>
       <c r="D299" t="inlineStr">
         <is>
-          <t>2026-08-09</t>
+          <t>2026-08-10</t>
         </is>
       </c>
     </row>
     <row r="300">
       <c r="A300" t="inlineStr">
         <is>
-          <t>キムさん</t>
+          <t>カー</t>
         </is>
       </c>
       <c r="B300" t="n">
@@ -49768,19 +50177,19 @@
       </c>
       <c r="C300" t="inlineStr">
         <is>
-          <t>2026-09-12</t>
+          <t>2026-08-09</t>
         </is>
       </c>
       <c r="D300" t="inlineStr">
         <is>
-          <t>2026-09-12</t>
+          <t>2026-08-09</t>
         </is>
       </c>
     </row>
     <row r="301">
       <c r="A301" t="inlineStr">
         <is>
-          <t>キムとどえむちゃん</t>
+          <t>キムさん</t>
         </is>
       </c>
       <c r="B301" t="n">
@@ -49788,19 +50197,19 @@
       </c>
       <c r="C301" t="inlineStr">
         <is>
-          <t>2026-08-20</t>
+          <t>2026-09-12</t>
         </is>
       </c>
       <c r="D301" t="inlineStr">
         <is>
-          <t>2026-08-20</t>
+          <t>2026-09-12</t>
         </is>
       </c>
     </row>
     <row r="302">
       <c r="A302" t="inlineStr">
         <is>
-          <t>キムとまゆ</t>
+          <t>キムとどえむちゃん</t>
         </is>
       </c>
       <c r="B302" t="n">
@@ -49808,19 +50217,19 @@
       </c>
       <c r="C302" t="inlineStr">
         <is>
-          <t>2026-09-08</t>
+          <t>2026-08-20</t>
         </is>
       </c>
       <c r="D302" t="inlineStr">
         <is>
-          <t>2026-09-08</t>
+          <t>2026-08-20</t>
         </is>
       </c>
     </row>
     <row r="303">
       <c r="A303" t="inlineStr">
         <is>
-          <t>キムとドM女R</t>
+          <t>キムとまゆ</t>
         </is>
       </c>
       <c r="B303" t="n">
@@ -49828,19 +50237,19 @@
       </c>
       <c r="C303" t="inlineStr">
         <is>
-          <t>2026-09-10</t>
+          <t>2026-09-08</t>
         </is>
       </c>
       <c r="D303" t="inlineStr">
         <is>
-          <t>2026-09-10</t>
+          <t>2026-09-08</t>
         </is>
       </c>
     </row>
     <row r="304">
       <c r="A304" t="inlineStr">
         <is>
-          <t>キムと奴隷</t>
+          <t>キムとドM女R</t>
         </is>
       </c>
       <c r="B304" t="n">
@@ -49848,19 +50257,19 @@
       </c>
       <c r="C304" t="inlineStr">
         <is>
-          <t>2026-08-16</t>
+          <t>2026-09-10</t>
         </is>
       </c>
       <c r="D304" t="inlineStr">
         <is>
-          <t>2026-08-16</t>
+          <t>2026-09-10</t>
         </is>
       </c>
     </row>
     <row r="305">
       <c r="A305" t="inlineStr">
         <is>
-          <t>キムと新しい奴隷ちゃん</t>
+          <t>キムと奴隷</t>
         </is>
       </c>
       <c r="B305" t="n">
@@ -49868,19 +50277,19 @@
       </c>
       <c r="C305" t="inlineStr">
         <is>
-          <t>2026-08-18</t>
+          <t>2026-08-16</t>
         </is>
       </c>
       <c r="D305" t="inlineStr">
         <is>
-          <t>2026-08-18</t>
+          <t>2026-08-16</t>
         </is>
       </c>
     </row>
     <row r="306">
       <c r="A306" t="inlineStr">
         <is>
-          <t>クロちゃん</t>
+          <t>キムと新しい奴隷ちゃん</t>
         </is>
       </c>
       <c r="B306" t="n">
@@ -49888,19 +50297,19 @@
       </c>
       <c r="C306" t="inlineStr">
         <is>
-          <t>2026-09-06</t>
+          <t>2026-08-18</t>
         </is>
       </c>
       <c r="D306" t="inlineStr">
         <is>
-          <t>2026-09-06</t>
+          <t>2026-08-18</t>
         </is>
       </c>
     </row>
     <row r="307">
       <c r="A307" t="inlineStr">
         <is>
-          <t>ケケ</t>
+          <t>クロちゃん</t>
         </is>
       </c>
       <c r="B307" t="n">
@@ -49920,7 +50329,7 @@
     <row r="308">
       <c r="A308" t="inlineStr">
         <is>
-          <t>ゲン</t>
+          <t>ケケ</t>
         </is>
       </c>
       <c r="B308" t="n">
@@ -49940,7 +50349,7 @@
     <row r="309">
       <c r="A309" t="inlineStr">
         <is>
-          <t>コオリ</t>
+          <t>ゲン</t>
         </is>
       </c>
       <c r="B309" t="n">
@@ -49948,19 +50357,19 @@
       </c>
       <c r="C309" t="inlineStr">
         <is>
-          <t>2026-08-11</t>
+          <t>2026-09-06</t>
         </is>
       </c>
       <c r="D309" t="inlineStr">
         <is>
-          <t>2026-08-11</t>
+          <t>2026-09-06</t>
         </is>
       </c>
     </row>
     <row r="310">
       <c r="A310" t="inlineStr">
         <is>
-          <t>サトル</t>
+          <t>コオリ</t>
         </is>
       </c>
       <c r="B310" t="n">
@@ -49968,19 +50377,19 @@
       </c>
       <c r="C310" t="inlineStr">
         <is>
-          <t>2026-09-11</t>
+          <t>2026-08-11</t>
         </is>
       </c>
       <c r="D310" t="inlineStr">
         <is>
-          <t>2026-09-11</t>
+          <t>2026-08-11</t>
         </is>
       </c>
     </row>
     <row r="311">
       <c r="A311" t="inlineStr">
         <is>
-          <t>ザッキー</t>
+          <t>サトル</t>
         </is>
       </c>
       <c r="B311" t="n">
@@ -49988,19 +50397,19 @@
       </c>
       <c r="C311" t="inlineStr">
         <is>
-          <t>2026-08-15</t>
+          <t>2026-09-11</t>
         </is>
       </c>
       <c r="D311" t="inlineStr">
         <is>
-          <t>2026-08-15</t>
+          <t>2026-09-11</t>
         </is>
       </c>
     </row>
     <row r="312">
       <c r="A312" t="inlineStr">
         <is>
-          <t>シゲ</t>
+          <t>ザッキー</t>
         </is>
       </c>
       <c r="B312" t="n">
@@ -50008,19 +50417,19 @@
       </c>
       <c r="C312" t="inlineStr">
         <is>
-          <t>2026-09-06</t>
+          <t>2026-08-15</t>
         </is>
       </c>
       <c r="D312" t="inlineStr">
         <is>
-          <t>2026-09-06</t>
+          <t>2026-08-15</t>
         </is>
       </c>
     </row>
     <row r="313">
       <c r="A313" t="inlineStr">
         <is>
-          <t>シュン</t>
+          <t>シゲ</t>
         </is>
       </c>
       <c r="B313" t="n">
@@ -50028,19 +50437,19 @@
       </c>
       <c r="C313" t="inlineStr">
         <is>
-          <t>2026-09-04</t>
+          <t>2026-09-06</t>
         </is>
       </c>
       <c r="D313" t="inlineStr">
         <is>
-          <t>2026-09-04</t>
+          <t>2026-09-06</t>
         </is>
       </c>
     </row>
     <row r="314">
       <c r="A314" t="inlineStr">
         <is>
-          <t>シュンヤ</t>
+          <t>シュン</t>
         </is>
       </c>
       <c r="B314" t="n">
@@ -50048,19 +50457,19 @@
       </c>
       <c r="C314" t="inlineStr">
         <is>
-          <t>2026-08-21</t>
+          <t>2026-09-04</t>
         </is>
       </c>
       <c r="D314" t="inlineStr">
         <is>
-          <t>2026-08-21</t>
+          <t>2026-09-04</t>
         </is>
       </c>
     </row>
     <row r="315">
       <c r="A315" t="inlineStr">
         <is>
-          <t>ジャッキー</t>
+          <t>シュンヤ</t>
         </is>
       </c>
       <c r="B315" t="n">
@@ -50068,19 +50477,19 @@
       </c>
       <c r="C315" t="inlineStr">
         <is>
-          <t>2026-08-29</t>
+          <t>2026-08-21</t>
         </is>
       </c>
       <c r="D315" t="inlineStr">
         <is>
-          <t>2026-08-29</t>
+          <t>2026-08-21</t>
         </is>
       </c>
     </row>
     <row r="316">
       <c r="A316" t="inlineStr">
         <is>
-          <t>ジョーカー</t>
+          <t>ジャッキー</t>
         </is>
       </c>
       <c r="B316" t="n">
@@ -50088,19 +50497,19 @@
       </c>
       <c r="C316" t="inlineStr">
         <is>
-          <t>2026-08-24</t>
+          <t>2026-08-29</t>
         </is>
       </c>
       <c r="D316" t="inlineStr">
         <is>
-          <t>2026-08-24</t>
+          <t>2026-08-29</t>
         </is>
       </c>
     </row>
     <row r="317">
       <c r="A317" t="inlineStr">
         <is>
-          <t>タカ</t>
+          <t>ジョーカー</t>
         </is>
       </c>
       <c r="B317" t="n">
@@ -50108,19 +50517,19 @@
       </c>
       <c r="C317" t="inlineStr">
         <is>
-          <t>2026-08-28</t>
+          <t>2026-08-24</t>
         </is>
       </c>
       <c r="D317" t="inlineStr">
         <is>
-          <t>2026-08-28</t>
+          <t>2026-08-24</t>
         </is>
       </c>
     </row>
     <row r="318">
       <c r="A318" t="inlineStr">
         <is>
-          <t>タカス</t>
+          <t>タカ</t>
         </is>
       </c>
       <c r="B318" t="n">
@@ -50128,19 +50537,19 @@
       </c>
       <c r="C318" t="inlineStr">
         <is>
-          <t>2026-08-18</t>
+          <t>2026-08-28</t>
         </is>
       </c>
       <c r="D318" t="inlineStr">
         <is>
-          <t>2026-08-18</t>
+          <t>2026-08-28</t>
         </is>
       </c>
     </row>
     <row r="319">
       <c r="A319" t="inlineStr">
         <is>
-          <t>タカ御一行</t>
+          <t>タカス</t>
         </is>
       </c>
       <c r="B319" t="n">
@@ -50148,19 +50557,19 @@
       </c>
       <c r="C319" t="inlineStr">
         <is>
-          <t>2026-09-12</t>
+          <t>2026-08-18</t>
         </is>
       </c>
       <c r="D319" t="inlineStr">
         <is>
-          <t>2026-09-12</t>
+          <t>2026-08-18</t>
         </is>
       </c>
     </row>
     <row r="320">
       <c r="A320" t="inlineStr">
         <is>
-          <t>ダイキ</t>
+          <t>タカ御一行</t>
         </is>
       </c>
       <c r="B320" t="n">
@@ -50168,19 +50577,19 @@
       </c>
       <c r="C320" t="inlineStr">
         <is>
-          <t>2026-08-25</t>
+          <t>2026-09-12</t>
         </is>
       </c>
       <c r="D320" t="inlineStr">
         <is>
-          <t>2026-08-25</t>
+          <t>2026-09-12</t>
         </is>
       </c>
     </row>
     <row r="321">
       <c r="A321" t="inlineStr">
         <is>
-          <t>ダイゴ</t>
+          <t>ダイキ</t>
         </is>
       </c>
       <c r="B321" t="n">
@@ -50188,19 +50597,19 @@
       </c>
       <c r="C321" t="inlineStr">
         <is>
-          <t>2026-08-21</t>
+          <t>2026-08-25</t>
         </is>
       </c>
       <c r="D321" t="inlineStr">
         <is>
-          <t>2026-08-21</t>
+          <t>2026-08-25</t>
         </is>
       </c>
     </row>
     <row r="322">
       <c r="A322" t="inlineStr">
         <is>
-          <t>ダイチ</t>
+          <t>ダイゴ</t>
         </is>
       </c>
       <c r="B322" t="n">
@@ -50208,19 +50617,19 @@
       </c>
       <c r="C322" t="inlineStr">
         <is>
-          <t>2026-08-11</t>
+          <t>2026-08-21</t>
         </is>
       </c>
       <c r="D322" t="inlineStr">
         <is>
-          <t>2026-08-11</t>
+          <t>2026-08-21</t>
         </is>
       </c>
     </row>
     <row r="323">
       <c r="A323" t="inlineStr">
         <is>
-          <t>ツシマ</t>
+          <t>ダイチ</t>
         </is>
       </c>
       <c r="B323" t="n">
@@ -50228,19 +50637,19 @@
       </c>
       <c r="C323" t="inlineStr">
         <is>
-          <t>2026-09-10</t>
+          <t>2026-08-11</t>
         </is>
       </c>
       <c r="D323" t="inlineStr">
         <is>
-          <t>2026-09-10</t>
+          <t>2026-08-11</t>
         </is>
       </c>
     </row>
     <row r="324">
       <c r="A324" t="inlineStr">
         <is>
-          <t>ツボ</t>
+          <t>ツシマ</t>
         </is>
       </c>
       <c r="B324" t="n">
@@ -50248,19 +50657,19 @@
       </c>
       <c r="C324" t="inlineStr">
         <is>
-          <t>2026-08-31</t>
+          <t>2026-09-10</t>
         </is>
       </c>
       <c r="D324" t="inlineStr">
         <is>
-          <t>2026-08-31</t>
+          <t>2026-09-10</t>
         </is>
       </c>
     </row>
     <row r="325">
       <c r="A325" t="inlineStr">
         <is>
-          <t>テクノっち</t>
+          <t>ツボ</t>
         </is>
       </c>
       <c r="B325" t="n">
@@ -50280,7 +50689,7 @@
     <row r="326">
       <c r="A326" t="inlineStr">
         <is>
-          <t>テクノとポチ</t>
+          <t>テクノっち</t>
         </is>
       </c>
       <c r="B326" t="n">
@@ -50288,19 +50697,19 @@
       </c>
       <c r="C326" t="inlineStr">
         <is>
-          <t>2026-08-12</t>
+          <t>2026-08-31</t>
         </is>
       </c>
       <c r="D326" t="inlineStr">
         <is>
-          <t>2026-08-12</t>
+          <t>2026-08-31</t>
         </is>
       </c>
     </row>
     <row r="327">
       <c r="A327" t="inlineStr">
         <is>
-          <t>テクノ＆てるくん＆イブオ</t>
+          <t>テクノとポチ</t>
         </is>
       </c>
       <c r="B327" t="n">
@@ -50308,19 +50717,19 @@
       </c>
       <c r="C327" t="inlineStr">
         <is>
-          <t>2026-09-06</t>
+          <t>2026-08-12</t>
         </is>
       </c>
       <c r="D327" t="inlineStr">
         <is>
-          <t>2026-09-06</t>
+          <t>2026-08-12</t>
         </is>
       </c>
     </row>
     <row r="328">
       <c r="A328" t="inlineStr">
         <is>
-          <t>トニー・トニー・チョッパー</t>
+          <t>テクノ＆てるくん＆イブオ</t>
         </is>
       </c>
       <c r="B328" t="n">
@@ -50328,19 +50737,19 @@
       </c>
       <c r="C328" t="inlineStr">
         <is>
-          <t>2026-08-23</t>
+          <t>2026-09-06</t>
         </is>
       </c>
       <c r="D328" t="inlineStr">
         <is>
-          <t>2026-08-23</t>
+          <t>2026-09-06</t>
         </is>
       </c>
     </row>
     <row r="329">
       <c r="A329" t="inlineStr">
         <is>
-          <t>ナカヤマヤ</t>
+          <t>トニー・トニー・チョッパー</t>
         </is>
       </c>
       <c r="B329" t="n">
@@ -50348,19 +50757,19 @@
       </c>
       <c r="C329" t="inlineStr">
         <is>
-          <t>2026-08-16</t>
+          <t>2026-08-23</t>
         </is>
       </c>
       <c r="D329" t="inlineStr">
         <is>
-          <t>2026-08-16</t>
+          <t>2026-08-23</t>
         </is>
       </c>
     </row>
     <row r="330">
       <c r="A330" t="inlineStr">
         <is>
-          <t>ニト</t>
+          <t>ナカヤマヤ</t>
         </is>
       </c>
       <c r="B330" t="n">
@@ -50368,19 +50777,19 @@
       </c>
       <c r="C330" t="inlineStr">
         <is>
-          <t>2026-08-27</t>
+          <t>2026-08-16</t>
         </is>
       </c>
       <c r="D330" t="inlineStr">
         <is>
-          <t>2026-08-27</t>
+          <t>2026-08-16</t>
         </is>
       </c>
     </row>
     <row r="331">
       <c r="A331" t="inlineStr">
         <is>
-          <t>ニャンまげ</t>
+          <t>ニト</t>
         </is>
       </c>
       <c r="B331" t="n">
@@ -50388,19 +50797,19 @@
       </c>
       <c r="C331" t="inlineStr">
         <is>
-          <t>2026-09-12</t>
+          <t>2026-08-27</t>
         </is>
       </c>
       <c r="D331" t="inlineStr">
         <is>
-          <t>2026-09-12</t>
+          <t>2026-08-27</t>
         </is>
       </c>
     </row>
     <row r="332">
       <c r="A332" t="inlineStr">
         <is>
-          <t>ビコー</t>
+          <t>ニャンまげ</t>
         </is>
       </c>
       <c r="B332" t="n">
@@ -50408,19 +50817,19 @@
       </c>
       <c r="C332" t="inlineStr">
         <is>
-          <t>2026-09-01</t>
+          <t>2026-09-12</t>
         </is>
       </c>
       <c r="D332" t="inlineStr">
         <is>
-          <t>2026-09-01</t>
+          <t>2026-09-12</t>
         </is>
       </c>
     </row>
     <row r="333">
       <c r="A333" t="inlineStr">
         <is>
-          <t>フジ</t>
+          <t>ビコー</t>
         </is>
       </c>
       <c r="B333" t="n">
@@ -50428,19 +50837,19 @@
       </c>
       <c r="C333" t="inlineStr">
         <is>
-          <t>2026-08-12</t>
+          <t>2026-09-01</t>
         </is>
       </c>
       <c r="D333" t="inlineStr">
         <is>
-          <t>2026-08-12</t>
+          <t>2026-09-01</t>
         </is>
       </c>
     </row>
     <row r="334">
       <c r="A334" t="inlineStr">
         <is>
-          <t>ボンタ</t>
+          <t>フジ</t>
         </is>
       </c>
       <c r="B334" t="n">
@@ -50448,19 +50857,19 @@
       </c>
       <c r="C334" t="inlineStr">
         <is>
-          <t>2026-08-10</t>
+          <t>2026-08-12</t>
         </is>
       </c>
       <c r="D334" t="inlineStr">
         <is>
-          <t>2026-08-10</t>
+          <t>2026-08-12</t>
         </is>
       </c>
     </row>
     <row r="335">
       <c r="A335" t="inlineStr">
         <is>
-          <t>ポチ</t>
+          <t>ボンタ</t>
         </is>
       </c>
       <c r="B335" t="n">
@@ -50468,19 +50877,19 @@
       </c>
       <c r="C335" t="inlineStr">
         <is>
-          <t>2026-09-06</t>
+          <t>2026-08-10</t>
         </is>
       </c>
       <c r="D335" t="inlineStr">
         <is>
-          <t>2026-09-06</t>
+          <t>2026-08-10</t>
         </is>
       </c>
     </row>
     <row r="336">
       <c r="A336" t="inlineStr">
         <is>
-          <t>マイナス</t>
+          <t>ポチ</t>
         </is>
       </c>
       <c r="B336" t="n">
@@ -50488,19 +50897,19 @@
       </c>
       <c r="C336" t="inlineStr">
         <is>
-          <t>2026-08-16</t>
+          <t>2026-09-06</t>
         </is>
       </c>
       <c r="D336" t="inlineStr">
         <is>
-          <t>2026-08-16</t>
+          <t>2026-09-06</t>
         </is>
       </c>
     </row>
     <row r="337">
       <c r="A337" t="inlineStr">
         <is>
-          <t>マサ</t>
+          <t>マイナス</t>
         </is>
       </c>
       <c r="B337" t="n">
@@ -50508,19 +50917,19 @@
       </c>
       <c r="C337" t="inlineStr">
         <is>
-          <t>2026-08-18</t>
+          <t>2026-08-16</t>
         </is>
       </c>
       <c r="D337" t="inlineStr">
         <is>
-          <t>2026-08-18</t>
+          <t>2026-08-16</t>
         </is>
       </c>
     </row>
     <row r="338">
       <c r="A338" t="inlineStr">
         <is>
-          <t>マッチョ</t>
+          <t>マサ</t>
         </is>
       </c>
       <c r="B338" t="n">
@@ -50528,19 +50937,19 @@
       </c>
       <c r="C338" t="inlineStr">
         <is>
-          <t>2026-08-10</t>
+          <t>2026-08-18</t>
         </is>
       </c>
       <c r="D338" t="inlineStr">
         <is>
-          <t>2026-08-10</t>
+          <t>2026-08-18</t>
         </is>
       </c>
     </row>
     <row r="339">
       <c r="A339" t="inlineStr">
         <is>
-          <t>マナティ</t>
+          <t>マッチョ</t>
         </is>
       </c>
       <c r="B339" t="n">
@@ -50548,19 +50957,19 @@
       </c>
       <c r="C339" t="inlineStr">
         <is>
-          <t>2026-08-12</t>
+          <t>2026-08-10</t>
         </is>
       </c>
       <c r="D339" t="inlineStr">
         <is>
-          <t>2026-08-12</t>
+          <t>2026-08-10</t>
         </is>
       </c>
     </row>
     <row r="340">
       <c r="A340" t="inlineStr">
         <is>
-          <t>ミスター工事マン</t>
+          <t>マナティ</t>
         </is>
       </c>
       <c r="B340" t="n">
@@ -50568,19 +50977,19 @@
       </c>
       <c r="C340" t="inlineStr">
         <is>
-          <t>2026-09-01</t>
+          <t>2026-08-12</t>
         </is>
       </c>
       <c r="D340" t="inlineStr">
         <is>
-          <t>2026-09-01</t>
+          <t>2026-08-12</t>
         </is>
       </c>
     </row>
     <row r="341">
       <c r="A341" t="inlineStr">
         <is>
-          <t>ミッシ</t>
+          <t>ミカミと仲間たち</t>
         </is>
       </c>
       <c r="B341" t="n">
@@ -50588,19 +50997,19 @@
       </c>
       <c r="C341" t="inlineStr">
         <is>
-          <t>2026-08-25</t>
+          <t>2026-09-15</t>
         </is>
       </c>
       <c r="D341" t="inlineStr">
         <is>
-          <t>2026-08-25</t>
+          <t>2026-09-15</t>
         </is>
       </c>
     </row>
     <row r="342">
       <c r="A342" t="inlineStr">
         <is>
-          <t>ミッチー</t>
+          <t>ミスター工事マン</t>
         </is>
       </c>
       <c r="B342" t="n">
@@ -50608,19 +51017,19 @@
       </c>
       <c r="C342" t="inlineStr">
         <is>
-          <t>2026-09-11</t>
+          <t>2026-09-01</t>
         </is>
       </c>
       <c r="D342" t="inlineStr">
         <is>
-          <t>2026-09-11</t>
+          <t>2026-09-01</t>
         </is>
       </c>
     </row>
     <row r="343">
       <c r="A343" t="inlineStr">
         <is>
-          <t>ミルコ</t>
+          <t>ミッシ</t>
         </is>
       </c>
       <c r="B343" t="n">
@@ -50628,19 +51037,19 @@
       </c>
       <c r="C343" t="inlineStr">
         <is>
-          <t>2026-09-11</t>
+          <t>2026-08-25</t>
         </is>
       </c>
       <c r="D343" t="inlineStr">
         <is>
-          <t>2026-09-11</t>
+          <t>2026-08-25</t>
         </is>
       </c>
     </row>
     <row r="344">
       <c r="A344" t="inlineStr">
         <is>
-          <t>モジャ</t>
+          <t>ミッチー</t>
         </is>
       </c>
       <c r="B344" t="n">
@@ -50648,19 +51057,19 @@
       </c>
       <c r="C344" t="inlineStr">
         <is>
-          <t>2026-08-26</t>
+          <t>2026-09-11</t>
         </is>
       </c>
       <c r="D344" t="inlineStr">
         <is>
-          <t>2026-08-26</t>
+          <t>2026-09-11</t>
         </is>
       </c>
     </row>
     <row r="345">
       <c r="A345" t="inlineStr">
         <is>
-          <t>ヤノちゃん</t>
+          <t>ミルコ</t>
         </is>
       </c>
       <c r="B345" t="n">
@@ -50668,19 +51077,19 @@
       </c>
       <c r="C345" t="inlineStr">
         <is>
-          <t>2026-09-04</t>
+          <t>2026-09-11</t>
         </is>
       </c>
       <c r="D345" t="inlineStr">
         <is>
-          <t>2026-09-04</t>
+          <t>2026-09-11</t>
         </is>
       </c>
     </row>
     <row r="346">
       <c r="A346" t="inlineStr">
         <is>
-          <t>ヤマ</t>
+          <t>モジャ</t>
         </is>
       </c>
       <c r="B346" t="n">
@@ -50688,19 +51097,19 @@
       </c>
       <c r="C346" t="inlineStr">
         <is>
-          <t>2026-09-07</t>
+          <t>2026-08-26</t>
         </is>
       </c>
       <c r="D346" t="inlineStr">
         <is>
-          <t>2026-09-07</t>
+          <t>2026-08-26</t>
         </is>
       </c>
     </row>
     <row r="347">
       <c r="A347" t="inlineStr">
         <is>
-          <t>ユウ</t>
+          <t>ヤノちゃん</t>
         </is>
       </c>
       <c r="B347" t="n">
@@ -50708,19 +51117,19 @@
       </c>
       <c r="C347" t="inlineStr">
         <is>
-          <t>2026-09-05</t>
+          <t>2026-09-04</t>
         </is>
       </c>
       <c r="D347" t="inlineStr">
         <is>
-          <t>2026-09-05</t>
+          <t>2026-09-04</t>
         </is>
       </c>
     </row>
     <row r="348">
       <c r="A348" t="inlineStr">
         <is>
-          <t>ユキ</t>
+          <t>ヤマ</t>
         </is>
       </c>
       <c r="B348" t="n">
@@ -50728,19 +51137,19 @@
       </c>
       <c r="C348" t="inlineStr">
         <is>
-          <t>2026-08-28</t>
+          <t>2026-09-07</t>
         </is>
       </c>
       <c r="D348" t="inlineStr">
         <is>
-          <t>2026-08-28</t>
+          <t>2026-09-07</t>
         </is>
       </c>
     </row>
     <row r="349">
       <c r="A349" t="inlineStr">
         <is>
-          <t>ユッキー</t>
+          <t>ユウ</t>
         </is>
       </c>
       <c r="B349" t="n">
@@ -50748,19 +51157,19 @@
       </c>
       <c r="C349" t="inlineStr">
         <is>
-          <t>2026-08-20</t>
+          <t>2026-09-05</t>
         </is>
       </c>
       <c r="D349" t="inlineStr">
         <is>
-          <t>2026-08-20</t>
+          <t>2026-09-05</t>
         </is>
       </c>
     </row>
     <row r="350">
       <c r="A350" t="inlineStr">
         <is>
-          <t>ヨシヤ</t>
+          <t>ユキ</t>
         </is>
       </c>
       <c r="B350" t="n">
@@ -50768,19 +51177,19 @@
       </c>
       <c r="C350" t="inlineStr">
         <is>
-          <t>2026-08-25</t>
+          <t>2026-08-28</t>
         </is>
       </c>
       <c r="D350" t="inlineStr">
         <is>
-          <t>2026-08-25</t>
+          <t>2026-08-28</t>
         </is>
       </c>
     </row>
     <row r="351">
       <c r="A351" t="inlineStr">
         <is>
-          <t>リク</t>
+          <t>ユッキー</t>
         </is>
       </c>
       <c r="B351" t="n">
@@ -50788,19 +51197,19 @@
       </c>
       <c r="C351" t="inlineStr">
         <is>
-          <t>2026-09-02</t>
+          <t>2026-08-20</t>
         </is>
       </c>
       <c r="D351" t="inlineStr">
         <is>
-          <t>2026-09-02</t>
+          <t>2026-08-20</t>
         </is>
       </c>
     </row>
     <row r="352">
       <c r="A352" t="inlineStr">
         <is>
-          <t>リョウ</t>
+          <t>ヨシヤ</t>
         </is>
       </c>
       <c r="B352" t="n">
@@ -50820,7 +51229,7 @@
     <row r="353">
       <c r="A353" t="inlineStr">
         <is>
-          <t>リン</t>
+          <t>リク</t>
         </is>
       </c>
       <c r="B353" t="n">
@@ -50828,19 +51237,19 @@
       </c>
       <c r="C353" t="inlineStr">
         <is>
-          <t>2026-09-03</t>
+          <t>2026-09-02</t>
         </is>
       </c>
       <c r="D353" t="inlineStr">
         <is>
-          <t>2026-09-03</t>
+          <t>2026-09-02</t>
         </is>
       </c>
     </row>
     <row r="354">
       <c r="A354" t="inlineStr">
         <is>
-          <t>ロタポジ</t>
+          <t>リョウ</t>
         </is>
       </c>
       <c r="B354" t="n">
@@ -50848,19 +51257,19 @@
       </c>
       <c r="C354" t="inlineStr">
         <is>
-          <t>2026-08-20</t>
+          <t>2026-08-25</t>
         </is>
       </c>
       <c r="D354" t="inlineStr">
         <is>
-          <t>2026-08-20</t>
+          <t>2026-08-25</t>
         </is>
       </c>
     </row>
     <row r="355">
       <c r="A355" t="inlineStr">
         <is>
-          <t>ローズ</t>
+          <t>リン</t>
         </is>
       </c>
       <c r="B355" t="n">
@@ -50868,19 +51277,19 @@
       </c>
       <c r="C355" t="inlineStr">
         <is>
-          <t>2026-09-12</t>
+          <t>2026-09-03</t>
         </is>
       </c>
       <c r="D355" t="inlineStr">
         <is>
-          <t>2026-09-12</t>
+          <t>2026-09-03</t>
         </is>
       </c>
     </row>
     <row r="356">
       <c r="A356" t="inlineStr">
         <is>
-          <t>僕と私</t>
+          <t>ロタポジ</t>
         </is>
       </c>
       <c r="B356" t="n">
@@ -50888,19 +51297,19 @@
       </c>
       <c r="C356" t="inlineStr">
         <is>
-          <t>2026-08-23</t>
+          <t>2026-08-20</t>
         </is>
       </c>
       <c r="D356" t="inlineStr">
         <is>
-          <t>2026-08-23</t>
+          <t>2026-08-20</t>
         </is>
       </c>
     </row>
     <row r="357">
       <c r="A357" t="inlineStr">
         <is>
-          <t>名無し</t>
+          <t>ローズ</t>
         </is>
       </c>
       <c r="B357" t="n">
@@ -50908,19 +51317,19 @@
       </c>
       <c r="C357" t="inlineStr">
         <is>
-          <t>2026-08-23</t>
+          <t>2026-09-12</t>
         </is>
       </c>
       <c r="D357" t="inlineStr">
         <is>
-          <t>2026-08-23</t>
+          <t>2026-09-12</t>
         </is>
       </c>
     </row>
     <row r="358">
       <c r="A358" t="inlineStr">
         <is>
-          <t>変態マッスル</t>
+          <t>僕と私</t>
         </is>
       </c>
       <c r="B358" t="n">
@@ -50928,19 +51337,19 @@
       </c>
       <c r="C358" t="inlineStr">
         <is>
-          <t>2026-09-12</t>
+          <t>2026-08-23</t>
         </is>
       </c>
       <c r="D358" t="inlineStr">
         <is>
-          <t>2026-09-12</t>
+          <t>2026-08-23</t>
         </is>
       </c>
     </row>
     <row r="359">
       <c r="A359" t="inlineStr">
         <is>
-          <t>大塚</t>
+          <t>名無し</t>
         </is>
       </c>
       <c r="B359" t="n">
@@ -50948,19 +51357,19 @@
       </c>
       <c r="C359" t="inlineStr">
         <is>
-          <t>2026-08-09</t>
+          <t>2026-08-23</t>
         </is>
       </c>
       <c r="D359" t="inlineStr">
         <is>
-          <t>2026-08-09</t>
+          <t>2026-08-23</t>
         </is>
       </c>
     </row>
     <row r="360">
       <c r="A360" t="inlineStr">
         <is>
-          <t>天我迅</t>
+          <t>変態マッスル</t>
         </is>
       </c>
       <c r="B360" t="n">
@@ -50968,19 +51377,19 @@
       </c>
       <c r="C360" t="inlineStr">
         <is>
-          <t>2026-09-09</t>
+          <t>2026-09-12</t>
         </is>
       </c>
       <c r="D360" t="inlineStr">
         <is>
-          <t>2026-09-09</t>
+          <t>2026-09-12</t>
         </is>
       </c>
     </row>
     <row r="361">
       <c r="A361" t="inlineStr">
         <is>
-          <t>女子三人衆</t>
+          <t>大塚</t>
         </is>
       </c>
       <c r="B361" t="n">
@@ -50988,19 +51397,19 @@
       </c>
       <c r="C361" t="inlineStr">
         <is>
-          <t>2026-08-16</t>
+          <t>2026-08-09</t>
         </is>
       </c>
       <c r="D361" t="inlineStr">
         <is>
-          <t>2026-08-16</t>
+          <t>2026-08-09</t>
         </is>
       </c>
     </row>
     <row r="362">
       <c r="A362" t="inlineStr">
         <is>
-          <t>正装しん</t>
+          <t>天我迅</t>
         </is>
       </c>
       <c r="B362" t="n">
@@ -51008,19 +51417,19 @@
       </c>
       <c r="C362" t="inlineStr">
         <is>
-          <t>2026-09-06</t>
+          <t>2026-09-09</t>
         </is>
       </c>
       <c r="D362" t="inlineStr">
         <is>
-          <t>2026-09-06</t>
+          <t>2026-09-09</t>
         </is>
       </c>
     </row>
     <row r="363">
       <c r="A363" t="inlineStr">
         <is>
-          <t>海砂利水魚</t>
+          <t>女子三人衆</t>
         </is>
       </c>
       <c r="B363" t="n">
@@ -51028,19 +51437,19 @@
       </c>
       <c r="C363" t="inlineStr">
         <is>
-          <t>2026-08-22</t>
+          <t>2026-08-16</t>
         </is>
       </c>
       <c r="D363" t="inlineStr">
         <is>
-          <t>2026-08-22</t>
+          <t>2026-08-16</t>
         </is>
       </c>
     </row>
     <row r="364">
       <c r="A364" t="inlineStr">
         <is>
-          <t>田中</t>
+          <t>正装しん</t>
         </is>
       </c>
       <c r="B364" t="n">
@@ -51048,19 +51457,19 @@
       </c>
       <c r="C364" t="inlineStr">
         <is>
-          <t>2026-09-05</t>
+          <t>2026-09-06</t>
         </is>
       </c>
       <c r="D364" t="inlineStr">
         <is>
-          <t>2026-09-05</t>
+          <t>2026-09-06</t>
         </is>
       </c>
     </row>
     <row r="365">
       <c r="A365" t="inlineStr">
         <is>
-          <t>番</t>
+          <t>海砂利水魚</t>
         </is>
       </c>
       <c r="B365" t="n">
@@ -51068,19 +51477,19 @@
       </c>
       <c r="C365" t="inlineStr">
         <is>
-          <t>2026-09-12</t>
+          <t>2026-08-22</t>
         </is>
       </c>
       <c r="D365" t="inlineStr">
         <is>
-          <t>2026-09-12</t>
+          <t>2026-08-22</t>
         </is>
       </c>
     </row>
     <row r="366">
       <c r="A366" t="inlineStr">
         <is>
-          <t>絶</t>
+          <t>田中</t>
         </is>
       </c>
       <c r="B366" t="n">
@@ -51088,19 +51497,19 @@
       </c>
       <c r="C366" t="inlineStr">
         <is>
-          <t>2026-08-15</t>
+          <t>2026-09-05</t>
         </is>
       </c>
       <c r="D366" t="inlineStr">
         <is>
-          <t>2026-08-15</t>
+          <t>2026-09-05</t>
         </is>
       </c>
     </row>
     <row r="367">
       <c r="A367" t="inlineStr">
         <is>
-          <t>絶ちゃん</t>
+          <t>番</t>
         </is>
       </c>
       <c r="B367" t="n">
@@ -51108,19 +51517,19 @@
       </c>
       <c r="C367" t="inlineStr">
         <is>
-          <t>2026-09-06</t>
+          <t>2026-09-12</t>
         </is>
       </c>
       <c r="D367" t="inlineStr">
         <is>
-          <t>2026-09-06</t>
+          <t>2026-09-12</t>
         </is>
       </c>
     </row>
     <row r="368">
       <c r="A368" t="inlineStr">
         <is>
-          <t>美優</t>
+          <t>絶</t>
         </is>
       </c>
       <c r="B368" t="n">
@@ -51128,19 +51537,19 @@
       </c>
       <c r="C368" t="inlineStr">
         <is>
-          <t>2026-09-09</t>
+          <t>2026-08-15</t>
         </is>
       </c>
       <c r="D368" t="inlineStr">
         <is>
-          <t>2026-09-09</t>
+          <t>2026-08-15</t>
         </is>
       </c>
     </row>
     <row r="369">
       <c r="A369" t="inlineStr">
         <is>
-          <t>赤ちゃん</t>
+          <t>絶ちゃん</t>
         </is>
       </c>
       <c r="B369" t="n">
@@ -51148,30 +51557,70 @@
       </c>
       <c r="C369" t="inlineStr">
         <is>
-          <t>2026-08-20</t>
+          <t>2026-09-06</t>
         </is>
       </c>
       <c r="D369" t="inlineStr">
         <is>
-          <t>2026-08-20</t>
+          <t>2026-09-06</t>
         </is>
       </c>
     </row>
     <row r="370">
       <c r="A370" t="inlineStr">
         <is>
+          <t>美優</t>
+        </is>
+      </c>
+      <c r="B370" t="n">
+        <v>1</v>
+      </c>
+      <c r="C370" t="inlineStr">
+        <is>
+          <t>2026-09-09</t>
+        </is>
+      </c>
+      <c r="D370" t="inlineStr">
+        <is>
+          <t>2026-09-09</t>
+        </is>
+      </c>
+    </row>
+    <row r="371">
+      <c r="A371" t="inlineStr">
+        <is>
+          <t>赤ちゃん</t>
+        </is>
+      </c>
+      <c r="B371" t="n">
+        <v>1</v>
+      </c>
+      <c r="C371" t="inlineStr">
+        <is>
+          <t>2026-08-20</t>
+        </is>
+      </c>
+      <c r="D371" t="inlineStr">
+        <is>
+          <t>2026-08-20</t>
+        </is>
+      </c>
+    </row>
+    <row r="372">
+      <c r="A372" t="inlineStr">
+        <is>
           <t>高田</t>
         </is>
       </c>
-      <c r="B370" t="n">
-        <v>1</v>
-      </c>
-      <c r="C370" t="inlineStr">
+      <c r="B372" t="n">
+        <v>1</v>
+      </c>
+      <c r="C372" t="inlineStr">
         <is>
           <t>2026-08-27</t>
         </is>
       </c>
-      <c r="D370" t="inlineStr">
+      <c r="D372" t="inlineStr">
         <is>
           <t>2026-08-27</t>
         </is>
@@ -51215,10 +51664,10 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>56</v>
+        <v>60</v>
       </c>
       <c r="C2" t="n">
-        <v>69</v>
+        <v>73</v>
       </c>
     </row>
     <row r="3">
@@ -51228,10 +51677,10 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="C3" t="n">
-        <v>70</v>
+        <v>71</v>
       </c>
     </row>
     <row r="4">
@@ -51363,10 +51812,10 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="C4" t="n">
-        <v>30</v>
+        <v>31</v>
       </c>
     </row>
     <row r="5">
@@ -51584,10 +52033,10 @@
         </is>
       </c>
       <c r="B21" t="n">
-        <v>82</v>
+        <v>85</v>
       </c>
       <c r="C21" t="n">
-        <v>97</v>
+        <v>100</v>
       </c>
     </row>
     <row r="22">
@@ -51597,10 +52046,10 @@
         </is>
       </c>
       <c r="B22" t="n">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="C22" t="n">
-        <v>78</v>
+        <v>79</v>
       </c>
     </row>
     <row r="23">
@@ -51701,13 +52150,13 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>159</v>
+        <v>164</v>
       </c>
       <c r="C3" t="n">
-        <v>198</v>
+        <v>203</v>
       </c>
       <c r="D3" t="n">
-        <v>151</v>
+        <v>153</v>
       </c>
     </row>
   </sheetData>

</xml_diff>